<commit_message>
Mass Upload Version 1: Working (Profit Center is Pending)
</commit_message>
<xml_diff>
--- a/app/initiator/webapp/templates/Cost Center Mass Upload Template.xlsx
+++ b/app/initiator/webapp/templates/Cost Center Mass Upload Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arjn\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E84858D-5CE3-49DE-95D7-145A56DB38DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5411F0FC-1CD7-43A1-BD22-F964E1EED3AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{014E9B38-2F05-48D9-BDF9-B41AF163D48F}"/>
   </bookViews>
@@ -14935,7 +14935,7 @@
           <x14:formula1>
             <xm:f>KPI!$C$2:$C$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:I1048576</xm:sqref>
+          <xm:sqref>H2:H1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0944667E-868D-4593-9672-88A5FC22CC7B}">
           <x14:formula1>

</xml_diff>